<commit_message>
Minor BOM edits #32
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.3/BOM/Client BOM IoT-Speaker v1.3.xlsx
+++ b/Design Files/IoT-Speaker-v1.3/BOM/Client BOM IoT-Speaker v1.3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Speaker-v1.3\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Speaker-v1.3\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -750,15 +750,9 @@
     <t>-</t>
   </si>
   <si>
-    <t>Adaptor</t>
-  </si>
-  <si>
     <t>Peripheral</t>
   </si>
   <si>
-    <t>Universal 5V 1A 2A Type C USB Charger Mobile Phone Wall Travel Power Adapter Charger EU/US Plug For Huawei Xiaomi iPhone Samsung ( 2A Rating Selected)</t>
-  </si>
-  <si>
     <t>Speaker</t>
   </si>
   <si>
@@ -775,12 +769,18 @@
   </si>
   <si>
     <t>803450 3.7V 1500mAh Lithium Polymer Rechargeable Battery For MP3 GPS Massager Camera Power Bank Laptop Speaker Lipo Li ion Cell</t>
+  </si>
+  <si>
+    <t>USB Cable</t>
+  </si>
+  <si>
+    <t>3A USB Type C Fast Charging Cable Quick Charger QC3.0 USB C Data Cable for Xiaomi Huawei Samsung Tablets Laptops 1M</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1448,7 +1448,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3598,7 +3598,7 @@
         <v>1</v>
       </c>
       <c r="L54" s="39">
-        <f t="shared" ref="L54:L56" si="22">K54*5</f>
+        <f t="shared" ref="L54:L57" si="22">K54*5</f>
         <v>5</v>
       </c>
       <c r="M54" s="38"/>
@@ -3610,19 +3610,19 @@
         <v>46</v>
       </c>
       <c r="C55" s="56" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E55" s="39" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F55" s="38" t="s">
         <v>242</v>
       </c>
       <c r="G55" s="39" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H55" s="64"/>
       <c r="I55" s="61"/>
@@ -3643,13 +3643,13 @@
         <v>47</v>
       </c>
       <c r="C56" s="57" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E56" s="39" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F56" s="38" t="s">
         <v>242</v>
@@ -3664,7 +3664,7 @@
         <v>242</v>
       </c>
       <c r="J56" s="62" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K56" s="60">
         <v>1</v>
@@ -3675,20 +3675,20 @@
       </c>
       <c r="M56" s="38"/>
     </row>
-    <row r="57" spans="1:13" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="50">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C57" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D57" s="38" t="s">
         <v>243</v>
       </c>
-      <c r="D57" s="38" t="s">
-        <v>244</v>
-      </c>
       <c r="E57" s="39" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F57" s="38" t="s">
         <v>242</v>
@@ -3701,13 +3701,14 @@
       </c>
       <c r="I57" s="36"/>
       <c r="J57" s="62" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K57" s="60">
         <v>1</v>
       </c>
       <c r="L57" s="39">
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>5</v>
       </c>
       <c r="M57" s="38"/>
     </row>

</xml_diff>

<commit_message>
#32 Client ,eSpark and JLCPCB BOM update acc to #31
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.3/BOM/Client BOM IoT-Speaker v1.3.xlsx
+++ b/Design Files/IoT-Speaker-v1.3/BOM/Client BOM IoT-Speaker v1.3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Speaker-v1.3\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Speaker-v1.3\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="257">
   <si>
     <t>Component list</t>
   </si>
@@ -201,9 +201,6 @@
     <t>R30, R32, R35, R39</t>
   </si>
   <si>
-    <t>R65</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -775,12 +772,30 @@
   </si>
   <si>
     <t>3A USB Type C Fast Charging Cable Quick Charger QC3.0 USB C Data Cable for Xiaomi Huawei Samsung Tablets Laptops 1M</t>
+  </si>
+  <si>
+    <t>R65, R69</t>
+  </si>
+  <si>
+    <t>C79</t>
+  </si>
+  <si>
+    <t>CAP CER 4700PF 1KV X7R 1206</t>
+  </si>
+  <si>
+    <t>Cap-1206</t>
+  </si>
+  <si>
+    <t>CC1206KKX7RCBB472</t>
+  </si>
+  <si>
+    <t>4.7nF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1448,7 +1463,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1746,7 +1761,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1787,7 +1802,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="52" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1806,7 +1821,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="53" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -1825,7 +1840,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -1911,31 +1926,31 @@
         <v>25</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H9" s="51" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>235</v>
+      </c>
+      <c r="J9" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="K9" s="58" t="s">
+        <v>234</v>
+      </c>
+      <c r="L9" s="51" t="s">
         <v>237</v>
       </c>
-      <c r="K9" s="58" t="s">
-        <v>235</v>
-      </c>
-      <c r="L9" s="51" t="s">
+      <c r="M9" s="29" t="s">
         <v>238</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1951,19 +1966,19 @@
         <v>26</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H10" s="63" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J10" s="36"/>
       <c r="K10" s="59">
@@ -1978,7 +1993,7 @@
     <row r="11" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B57" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B58" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="56" t="s">
@@ -1988,19 +2003,19 @@
         <v>27</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H11" s="64" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J11" s="38"/>
       <c r="K11" s="60">
@@ -2025,19 +2040,19 @@
         <v>28</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H12" s="63" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J12" s="36"/>
       <c r="K12" s="59">
@@ -2062,19 +2077,19 @@
         <v>29</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H13" s="64" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J13" s="38"/>
       <c r="K13" s="60">
@@ -2099,19 +2114,19 @@
         <v>30</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H14" s="63" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J14" s="36"/>
       <c r="K14" s="59">
@@ -2136,26 +2151,26 @@
         <v>31</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H15" s="64" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J15" s="38"/>
       <c r="K15" s="60">
         <v>4</v>
       </c>
       <c r="L15" s="39">
-        <f t="shared" ref="L15" si="3">K15*5</f>
+        <f t="shared" ref="L15:L16" si="3">K15*5</f>
         <v>20</v>
       </c>
       <c r="M15" s="38"/>
@@ -2163,1514 +2178,1512 @@
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="50">
-        <f>ROW(B16) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="55" t="s">
-        <v>8</v>
+      <c r="C16" s="57" t="s">
+        <v>7</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" s="37" t="s">
-        <v>78</v>
+        <v>252</v>
+      </c>
+      <c r="E16" s="36" t="s">
+        <v>253</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="G16" s="37" t="s">
-        <v>156</v>
-      </c>
-      <c r="H16" s="63" t="s">
-        <v>191</v>
+        <v>254</v>
+      </c>
+      <c r="G16" s="36" t="s">
+        <v>255</v>
+      </c>
+      <c r="H16" s="36" t="s">
+        <v>189</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="J16" s="36"/>
       <c r="K16" s="59">
         <v>1</v>
       </c>
       <c r="L16" s="37">
-        <f>K16*5</f>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="M16" s="36"/>
     </row>
-    <row r="17" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
       <c r="C17" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="D17" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>122</v>
-      </c>
-      <c r="G17" s="39" t="s">
-        <v>157</v>
-      </c>
-      <c r="H17" s="64" t="s">
-        <v>192</v>
+      <c r="D17" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="H17" s="63" t="s">
+        <v>190</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J17" s="36"/>
-      <c r="K17" s="60">
+      <c r="K17" s="59">
         <v>1</v>
       </c>
-      <c r="L17" s="39">
-        <f t="shared" ref="L17" si="4">K17*5</f>
+      <c r="L17" s="37">
+        <f>K17*5</f>
         <v>5</v>
       </c>
-      <c r="M17" s="38"/>
+      <c r="M17" s="36"/>
     </row>
     <row r="18" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
-        <f>ROW(B18) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="36" t="s">
-        <v>34</v>
-      </c>
-      <c r="E18" s="37" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="H18" s="63" t="s">
-        <v>193</v>
+        <v>8</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>156</v>
+      </c>
+      <c r="H18" s="64" t="s">
+        <v>191</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J18" s="36"/>
-      <c r="K18" s="59">
+      <c r="K18" s="60">
         <v>1</v>
       </c>
-      <c r="L18" s="37">
-        <f>K18*5</f>
+      <c r="L18" s="39">
+        <f t="shared" ref="L18" si="4">K18*5</f>
         <v>5</v>
       </c>
-      <c r="M18" s="36"/>
-    </row>
-    <row r="19" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M18" s="38"/>
+    </row>
+    <row r="19" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="56" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="F19" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="H19" s="64" t="s">
-        <v>194</v>
+      <c r="C19" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="G19" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="H19" s="63" t="s">
+        <v>192</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J19" s="36"/>
-      <c r="K19" s="60">
-        <v>3</v>
-      </c>
-      <c r="L19" s="39">
-        <f t="shared" ref="L19" si="5">K19*5</f>
-        <v>15</v>
-      </c>
-      <c r="M19" s="38"/>
-    </row>
-    <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K19" s="59">
+        <v>1</v>
+      </c>
+      <c r="L19" s="37">
+        <f>K19*5</f>
+        <v>5</v>
+      </c>
+      <c r="M19" s="36"/>
+    </row>
+    <row r="20" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
-        <f>ROW(B20) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="55" t="s">
+      <c r="C20" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="G20" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="H20" s="63" t="s">
-        <v>194</v>
+      <c r="D20" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="H20" s="64" t="s">
+        <v>193</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J20" s="36"/>
-      <c r="K20" s="59">
-        <v>1</v>
-      </c>
-      <c r="L20" s="37">
-        <f>K20*5</f>
-        <v>5</v>
-      </c>
-      <c r="M20" s="36"/>
-    </row>
-    <row r="21" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="60">
+        <v>3</v>
+      </c>
+      <c r="L20" s="39">
+        <f t="shared" ref="L20" si="5">K20*5</f>
+        <v>15</v>
+      </c>
+      <c r="M20" s="38"/>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="56" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="38" t="s">
-        <v>37</v>
-      </c>
-      <c r="E21" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="G21" s="39" t="s">
-        <v>161</v>
-      </c>
-      <c r="H21" s="64" t="s">
-        <v>195</v>
+      <c r="C21" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="H21" s="63" t="s">
+        <v>193</v>
       </c>
       <c r="I21" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J21" s="36"/>
-      <c r="K21" s="60">
+      <c r="K21" s="59">
         <v>1</v>
       </c>
-      <c r="L21" s="39">
-        <f t="shared" ref="L21" si="6">K21*5</f>
+      <c r="L21" s="37">
+        <f>K21*5</f>
         <v>5</v>
       </c>
-      <c r="M21" s="38"/>
-    </row>
-    <row r="22" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M21" s="36"/>
+    </row>
+    <row r="22" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="37" t="s">
-        <v>84</v>
-      </c>
-      <c r="F22" s="36" t="s">
-        <v>127</v>
-      </c>
-      <c r="G22" s="37" t="s">
-        <v>162</v>
-      </c>
-      <c r="H22" s="63" t="s">
-        <v>196</v>
+      <c r="C22" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="H22" s="64" t="s">
+        <v>194</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J22" s="36"/>
-      <c r="K22" s="59">
+      <c r="K22" s="60">
         <v>1</v>
       </c>
-      <c r="L22" s="37">
-        <f>K22*5</f>
+      <c r="L22" s="39">
+        <f t="shared" ref="L22" si="6">K22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="36"/>
-    </row>
-    <row r="23" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M22" s="38"/>
+    </row>
+    <row r="23" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="56" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="E23" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="G23" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="H23" s="64" t="s">
-        <v>197</v>
+      <c r="C23" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="G23" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="H23" s="63" t="s">
+        <v>195</v>
       </c>
       <c r="I23" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J23" s="36"/>
-      <c r="K23" s="60">
+      <c r="K23" s="59">
         <v>1</v>
       </c>
-      <c r="L23" s="39">
-        <f t="shared" ref="L23" si="7">K23*5</f>
+      <c r="L23" s="37">
+        <f>K23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="38"/>
-    </row>
-    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M23" s="36"/>
+    </row>
+    <row r="24" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
-        <f>ROW(B24) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="F24" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="G24" s="37">
-        <v>61300211121</v>
-      </c>
-      <c r="H24" s="63" t="s">
-        <v>198</v>
+      <c r="C24" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="G24" s="39" t="s">
+        <v>162</v>
+      </c>
+      <c r="H24" s="64" t="s">
+        <v>196</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J24" s="36"/>
-      <c r="K24" s="59">
+      <c r="K24" s="60">
         <v>1</v>
       </c>
-      <c r="L24" s="37">
-        <f>K24*5</f>
+      <c r="L24" s="39">
+        <f t="shared" ref="L24" si="7">K24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="36"/>
-    </row>
-    <row r="25" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M24" s="38"/>
+    </row>
+    <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="56" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="G25" s="39" t="s">
-        <v>130</v>
-      </c>
-      <c r="H25" s="64" t="s">
-        <v>199</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>221</v>
-      </c>
-      <c r="J25" s="38"/>
-      <c r="K25" s="60">
+      <c r="C25" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="G25" s="37">
+        <v>61300211121</v>
+      </c>
+      <c r="H25" s="63" t="s">
+        <v>197</v>
+      </c>
+      <c r="I25" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="J25" s="36"/>
+      <c r="K25" s="59">
         <v>1</v>
       </c>
-      <c r="L25" s="39">
-        <f t="shared" ref="L25" si="8">K25*5</f>
+      <c r="L25" s="37">
+        <f>K25*5</f>
         <v>5</v>
       </c>
-      <c r="M25" s="38"/>
+      <c r="M25" s="36"/>
     </row>
     <row r="26" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
-        <f>ROW(B26) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="55" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="F26" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="G26" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="H26" s="63" t="s">
-        <v>200</v>
-      </c>
-      <c r="I26" s="36" t="s">
-        <v>222</v>
-      </c>
-      <c r="J26" s="36"/>
-      <c r="K26" s="59">
-        <v>2</v>
-      </c>
-      <c r="L26" s="37">
-        <f>K26*5</f>
-        <v>10</v>
-      </c>
-      <c r="M26" s="36"/>
+      <c r="C26" s="56" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="G26" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="I26" s="38" t="s">
+        <v>220</v>
+      </c>
+      <c r="J26" s="38"/>
+      <c r="K26" s="60">
+        <v>1</v>
+      </c>
+      <c r="L26" s="39">
+        <f t="shared" ref="L26" si="8">K26*5</f>
+        <v>5</v>
+      </c>
+      <c r="M26" s="38"/>
     </row>
     <row r="27" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="56" t="s">
-        <v>17</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="E27" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="F27" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="G27" s="39" t="s">
-        <v>164</v>
-      </c>
-      <c r="H27" s="64" t="s">
-        <v>201</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>242</v>
-      </c>
-      <c r="J27" s="38"/>
-      <c r="K27" s="60">
-        <v>1</v>
-      </c>
-      <c r="L27" s="39">
-        <f t="shared" ref="L27" si="9">K27*5</f>
-        <v>5</v>
-      </c>
-      <c r="M27" s="38"/>
+      <c r="C27" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="F27" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="G27" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="H27" s="63" t="s">
+        <v>199</v>
+      </c>
+      <c r="I27" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="J27" s="36"/>
+      <c r="K27" s="59">
+        <v>2</v>
+      </c>
+      <c r="L27" s="37">
+        <f>K27*5</f>
+        <v>10</v>
+      </c>
+      <c r="M27" s="36"/>
     </row>
     <row r="28" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
-        <f>ROW(B28) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="G28" s="37" t="s">
-        <v>133</v>
-      </c>
-      <c r="H28" s="63" t="s">
-        <v>202</v>
-      </c>
-      <c r="I28" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="J28" s="36"/>
-      <c r="K28" s="59">
-        <v>3</v>
-      </c>
-      <c r="L28" s="37">
-        <f>K28*5</f>
-        <v>15</v>
-      </c>
-      <c r="M28" s="36"/>
-    </row>
-    <row r="29" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="56" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>131</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="H28" s="64" t="s">
+        <v>200</v>
+      </c>
+      <c r="I28" s="38" t="s">
+        <v>241</v>
+      </c>
+      <c r="J28" s="38"/>
+      <c r="K28" s="60">
+        <v>1</v>
+      </c>
+      <c r="L28" s="39">
+        <f t="shared" ref="L28" si="9">K28*5</f>
+        <v>5</v>
+      </c>
+      <c r="M28" s="38"/>
+    </row>
+    <row r="29" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
       <c r="C29" s="55" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G29" s="37" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="H29" s="63" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I29" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J29" s="36"/>
       <c r="K29" s="59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L29" s="37">
         <f>K29*5</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="M29" s="36"/>
     </row>
-    <row r="30" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="56" t="s">
+      <c r="C30" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="D30" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="E30" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="38" t="s">
-        <v>135</v>
-      </c>
-      <c r="G30" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="H30" s="64" t="s">
-        <v>204</v>
+      <c r="D30" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="H30" s="63" t="s">
+        <v>202</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J30" s="36"/>
-      <c r="K30" s="60">
-        <v>2</v>
-      </c>
-      <c r="L30" s="39">
-        <f t="shared" ref="L30" si="10">K30*5</f>
-        <v>10</v>
-      </c>
-      <c r="M30" s="38"/>
-    </row>
-    <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="59">
+        <v>1</v>
+      </c>
+      <c r="L30" s="37">
+        <f>K30*5</f>
+        <v>5</v>
+      </c>
+      <c r="M30" s="36"/>
+    </row>
+    <row r="31" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
-        <f>ROW(B31) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="55" t="s">
+      <c r="C31" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="E31" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="F31" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="G31" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="H31" s="63" t="s">
-        <v>204</v>
+      <c r="D31" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="G31" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="H31" s="64" t="s">
+        <v>203</v>
       </c>
       <c r="I31" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J31" s="36"/>
-      <c r="K31" s="59">
-        <v>1</v>
-      </c>
-      <c r="L31" s="37">
-        <f>K31*5</f>
-        <v>5</v>
-      </c>
-      <c r="M31" s="36"/>
+      <c r="K31" s="60">
+        <v>2</v>
+      </c>
+      <c r="L31" s="39">
+        <f t="shared" ref="L31" si="10">K31*5</f>
+        <v>10</v>
+      </c>
+      <c r="M31" s="38"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="56" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="F32" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="H32" s="64" t="s">
-        <v>190</v>
-      </c>
-      <c r="I32" s="38" t="s">
-        <v>223</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="60">
-        <v>2</v>
-      </c>
-      <c r="L32" s="39">
-        <f t="shared" ref="L32" si="11">K32*5</f>
-        <v>10</v>
-      </c>
-      <c r="M32" s="38"/>
+      <c r="C32" s="55" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="H32" s="63" t="s">
+        <v>203</v>
+      </c>
+      <c r="I32" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="J32" s="36"/>
+      <c r="K32" s="59">
+        <v>1</v>
+      </c>
+      <c r="L32" s="37">
+        <f>K32*5</f>
+        <v>5</v>
+      </c>
+      <c r="M32" s="36"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="55" t="s">
+      <c r="C33" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="D33" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="E33" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="F33" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="G33" s="37" t="s">
-        <v>169</v>
-      </c>
-      <c r="H33" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I33" s="36" t="s">
-        <v>224</v>
-      </c>
-      <c r="J33" s="36"/>
-      <c r="K33" s="59">
-        <v>1</v>
-      </c>
-      <c r="L33" s="37">
-        <f>K33*5</f>
-        <v>5</v>
-      </c>
-      <c r="M33" s="36"/>
-    </row>
-    <row r="34" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G33" s="39" t="s">
+        <v>167</v>
+      </c>
+      <c r="H33" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="I33" s="38" t="s">
+        <v>222</v>
+      </c>
+      <c r="J33" s="38"/>
+      <c r="K33" s="60">
+        <v>2</v>
+      </c>
+      <c r="L33" s="39">
+        <f t="shared" ref="L33" si="11">K33*5</f>
+        <v>10</v>
+      </c>
+      <c r="M33" s="38"/>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="56" t="s">
+      <c r="C34" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D34" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="E34" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="F34" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="G34" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="H34" s="64" t="s">
-        <v>205</v>
-      </c>
-      <c r="I34" s="38" t="s">
-        <v>225</v>
-      </c>
-      <c r="J34" s="38"/>
-      <c r="K34" s="60">
+      <c r="D34" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="F34" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="H34" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I34" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="J34" s="36"/>
+      <c r="K34" s="59">
         <v>1</v>
       </c>
-      <c r="L34" s="39">
-        <f t="shared" ref="L34" si="12">K34*5</f>
+      <c r="L34" s="37">
+        <f>K34*5</f>
         <v>5</v>
       </c>
-      <c r="M34" s="38"/>
-    </row>
-    <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M34" s="36"/>
+    </row>
+    <row r="35" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
-        <f>ROW(B35) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="55" t="s">
+      <c r="C35" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="D35" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="E35" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="F35" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="G35" s="37" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="J35" s="36"/>
-      <c r="K35" s="59">
-        <v>6</v>
-      </c>
-      <c r="L35" s="37">
-        <f>K35*5</f>
-        <v>30</v>
-      </c>
-      <c r="M35" s="36"/>
-    </row>
-    <row r="36" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D35" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="F35" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G35" s="39" t="s">
+        <v>169</v>
+      </c>
+      <c r="H35" s="64" t="s">
+        <v>204</v>
+      </c>
+      <c r="I35" s="38" t="s">
+        <v>224</v>
+      </c>
+      <c r="J35" s="38"/>
+      <c r="K35" s="60">
+        <v>1</v>
+      </c>
+      <c r="L35" s="39">
+        <f t="shared" ref="L35" si="12">K35*5</f>
+        <v>5</v>
+      </c>
+      <c r="M35" s="38"/>
+    </row>
+    <row r="36" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="56" t="s">
+      <c r="C36" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D36" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="E36" s="39" t="s">
-        <v>98</v>
-      </c>
-      <c r="F36" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="G36" s="39" t="s">
-        <v>172</v>
-      </c>
-      <c r="H36" s="64" t="s">
-        <v>206</v>
-      </c>
-      <c r="I36" s="38" t="s">
-        <v>227</v>
-      </c>
-      <c r="J36" s="38"/>
-      <c r="K36" s="60">
-        <v>1</v>
-      </c>
-      <c r="L36" s="39">
-        <f t="shared" ref="L36" si="13">K36*5</f>
-        <v>5</v>
-      </c>
-      <c r="M36" s="38"/>
-    </row>
-    <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D36" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="F36" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="H36" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I36" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="J36" s="36"/>
+      <c r="K36" s="59">
+        <v>6</v>
+      </c>
+      <c r="L36" s="37">
+        <f>K36*5</f>
+        <v>30</v>
+      </c>
+      <c r="M36" s="36"/>
+    </row>
+    <row r="37" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
-        <f>ROW(B37) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="55" t="s">
+      <c r="C37" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="E37" s="37" t="s">
-        <v>99</v>
-      </c>
-      <c r="F37" s="36" t="s">
+      <c r="D37" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F37" s="38" t="s">
         <v>137</v>
       </c>
-      <c r="G37" s="37" t="s">
-        <v>173</v>
-      </c>
-      <c r="H37" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I37" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="J37" s="36"/>
-      <c r="K37" s="59">
-        <v>3</v>
-      </c>
-      <c r="L37" s="37">
-        <f>K37*5</f>
-        <v>15</v>
-      </c>
-      <c r="M37" s="36"/>
+      <c r="G37" s="39" t="s">
+        <v>171</v>
+      </c>
+      <c r="H37" s="64" t="s">
+        <v>205</v>
+      </c>
+      <c r="I37" s="38" t="s">
+        <v>226</v>
+      </c>
+      <c r="J37" s="38"/>
+      <c r="K37" s="60">
+        <v>1</v>
+      </c>
+      <c r="L37" s="39">
+        <f t="shared" ref="L37" si="13">K37*5</f>
+        <v>5</v>
+      </c>
+      <c r="M37" s="38"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D38" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="E38" s="39" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="G38" s="39" t="s">
-        <v>174</v>
-      </c>
-      <c r="H38" s="64" t="s">
-        <v>190</v>
-      </c>
-      <c r="I38" s="38" t="s">
-        <v>229</v>
-      </c>
-      <c r="J38" s="38"/>
-      <c r="K38" s="60">
+      <c r="D38" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="F38" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="H38" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I38" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="J38" s="36"/>
+      <c r="K38" s="59">
         <v>3</v>
       </c>
-      <c r="L38" s="39">
-        <f t="shared" ref="L38" si="14">K38*5</f>
+      <c r="L38" s="37">
+        <f>K38*5</f>
         <v>15</v>
       </c>
-      <c r="M38" s="38"/>
+      <c r="M38" s="36"/>
     </row>
     <row r="39" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="50">
-        <f>ROW(B39) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D39" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" s="37" t="s">
-        <v>101</v>
-      </c>
-      <c r="F39" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="G39" s="37" t="s">
-        <v>175</v>
-      </c>
-      <c r="H39" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I39" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="J39" s="36"/>
-      <c r="K39" s="59">
+      <c r="D39" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="E39" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="F39" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G39" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="H39" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="I39" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="J39" s="38"/>
+      <c r="K39" s="60">
         <v>3</v>
       </c>
-      <c r="L39" s="37">
-        <f>K39*5</f>
+      <c r="L39" s="39">
+        <f t="shared" ref="L39" si="14">K39*5</f>
         <v>15</v>
       </c>
-      <c r="M39" s="36"/>
+      <c r="M39" s="38"/>
     </row>
     <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D40" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="E40" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="F40" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="G40" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="H40" s="64" t="s">
-        <v>207</v>
-      </c>
-      <c r="I40" s="38" t="s">
-        <v>231</v>
-      </c>
-      <c r="J40" s="38"/>
-      <c r="K40" s="60">
-        <v>4</v>
-      </c>
-      <c r="L40" s="39">
-        <f t="shared" ref="L40" si="15">K40*5</f>
-        <v>20</v>
-      </c>
-      <c r="M40" s="38"/>
+      <c r="D40" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="F40" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G40" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="H40" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I40" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="J40" s="36"/>
+      <c r="K40" s="59">
+        <v>3</v>
+      </c>
+      <c r="L40" s="37">
+        <f>K40*5</f>
+        <v>15</v>
+      </c>
+      <c r="M40" s="36"/>
     </row>
     <row r="41" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="50">
-        <f>ROW(B41) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D41" s="36" t="s">
-        <v>57</v>
-      </c>
-      <c r="E41" s="37" t="s">
-        <v>103</v>
-      </c>
-      <c r="F41" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="G41" s="37" t="s">
-        <v>177</v>
-      </c>
-      <c r="H41" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I41" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="J41" s="36"/>
-      <c r="K41" s="59">
-        <v>2</v>
-      </c>
-      <c r="L41" s="37">
-        <f>K41*5</f>
-        <v>10</v>
-      </c>
-      <c r="M41" s="36"/>
+      <c r="D41" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="F41" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="G41" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="H41" s="64" t="s">
+        <v>206</v>
+      </c>
+      <c r="I41" s="38" t="s">
+        <v>230</v>
+      </c>
+      <c r="J41" s="38"/>
+      <c r="K41" s="60">
+        <v>4</v>
+      </c>
+      <c r="L41" s="39">
+        <f t="shared" ref="L41" si="15">K41*5</f>
+        <v>20</v>
+      </c>
+      <c r="M41" s="38"/>
     </row>
     <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="56" t="s">
+      <c r="C42" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="E42" s="39" t="s">
-        <v>104</v>
-      </c>
-      <c r="F42" s="38" t="s">
+      <c r="D42" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="E42" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="F42" s="36" t="s">
         <v>137</v>
       </c>
-      <c r="G42" s="39" t="s">
-        <v>178</v>
-      </c>
-      <c r="H42" s="64" t="s">
-        <v>190</v>
-      </c>
-      <c r="I42" s="38" t="s">
-        <v>232</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="60">
+      <c r="G42" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="H42" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I42" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="J42" s="36"/>
+      <c r="K42" s="59">
         <v>2</v>
       </c>
-      <c r="L42" s="39">
-        <f t="shared" ref="L42" si="16">K42*5</f>
+      <c r="L42" s="37">
+        <f>K42*5</f>
         <v>10</v>
       </c>
-      <c r="M42" s="38"/>
+      <c r="M42" s="36"/>
     </row>
     <row r="43" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="50">
-        <f>ROW(B43) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="55" t="s">
+      <c r="C43" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="D43" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="E43" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="F43" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="G43" s="37" t="s">
-        <v>179</v>
-      </c>
-      <c r="H43" s="63" t="s">
-        <v>190</v>
-      </c>
-      <c r="I43" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="J43" s="36"/>
-      <c r="K43" s="59">
-        <v>4</v>
-      </c>
-      <c r="L43" s="37">
-        <f>K43*5</f>
-        <v>20</v>
-      </c>
-      <c r="M43" s="36"/>
+      <c r="D43" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="E43" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F43" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G43" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="H43" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="I43" s="38" t="s">
+        <v>231</v>
+      </c>
+      <c r="J43" s="38"/>
+      <c r="K43" s="60">
+        <v>2</v>
+      </c>
+      <c r="L43" s="39">
+        <f t="shared" ref="L43" si="16">K43*5</f>
+        <v>10</v>
+      </c>
+      <c r="M43" s="38"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
       <c r="C44" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D44" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="E44" s="39" t="s">
-        <v>106</v>
-      </c>
-      <c r="F44" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="G44" s="39" t="s">
-        <v>180</v>
-      </c>
-      <c r="H44" s="64" t="s">
-        <v>190</v>
-      </c>
-      <c r="I44" s="38" t="s">
-        <v>234</v>
-      </c>
-      <c r="J44" s="38"/>
-      <c r="K44" s="60">
-        <v>1</v>
-      </c>
-      <c r="L44" s="39">
-        <f t="shared" ref="L44" si="17">K44*5</f>
-        <v>5</v>
-      </c>
-      <c r="M44" s="38"/>
-    </row>
-    <row r="45" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D44" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="E44" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="F44" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G44" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="H44" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="I44" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="J44" s="36"/>
+      <c r="K44" s="59">
+        <v>4</v>
+      </c>
+      <c r="L44" s="37">
+        <f>K44*5</f>
+        <v>20</v>
+      </c>
+      <c r="M44" s="36"/>
+    </row>
+    <row r="45" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="50">
-        <f>ROW(B45) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C45" s="55" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D45" s="36" t="s">
-        <v>61</v>
-      </c>
-      <c r="E45" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="F45" s="36" t="s">
-        <v>139</v>
-      </c>
-      <c r="G45" s="37" t="s">
-        <v>139</v>
-      </c>
-      <c r="H45" s="63" t="s">
-        <v>208</v>
-      </c>
-      <c r="I45" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="J45" s="36"/>
-      <c r="K45" s="59">
-        <v>1</v>
-      </c>
-      <c r="L45" s="37">
-        <f>K45*5</f>
-        <v>5</v>
-      </c>
-      <c r="M45" s="36"/>
-    </row>
-    <row r="46" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>251</v>
+      </c>
+      <c r="E45" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="F45" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G45" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="H45" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="I45" s="38" t="s">
+        <v>233</v>
+      </c>
+      <c r="J45" s="38"/>
+      <c r="K45" s="60">
+        <v>2</v>
+      </c>
+      <c r="L45" s="39">
+        <f t="shared" ref="L45" si="17">K45*5</f>
+        <v>10</v>
+      </c>
+      <c r="M45" s="38"/>
+    </row>
+    <row r="46" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="D46" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="E46" s="39" t="s">
-        <v>108</v>
-      </c>
-      <c r="F46" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="G46" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="H46" s="64" t="s">
-        <v>209</v>
+      <c r="C46" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="E46" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="F46" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="G46" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="H46" s="63" t="s">
+        <v>207</v>
       </c>
       <c r="I46" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J46" s="36"/>
-      <c r="K46" s="60">
-        <v>4</v>
-      </c>
-      <c r="L46" s="39">
-        <f t="shared" ref="L46" si="18">K46*5</f>
-        <v>20</v>
-      </c>
-      <c r="M46" s="38"/>
-    </row>
-    <row r="47" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K46" s="59">
+        <v>1</v>
+      </c>
+      <c r="L46" s="37">
+        <f>K46*5</f>
+        <v>5</v>
+      </c>
+      <c r="M46" s="36"/>
+    </row>
+    <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="50">
-        <f>ROW(B47) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="D47" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="E47" s="37" t="s">
-        <v>109</v>
-      </c>
-      <c r="F47" s="36" t="s">
-        <v>141</v>
-      </c>
-      <c r="G47" s="37" t="s">
-        <v>181</v>
-      </c>
-      <c r="H47" s="63" t="s">
+      <c r="C47" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E47" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F47" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="G47" s="39" t="s">
+        <v>139</v>
+      </c>
+      <c r="H47" s="64" t="s">
         <v>208</v>
       </c>
       <c r="I47" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J47" s="36"/>
-      <c r="K47" s="59">
-        <v>1</v>
-      </c>
-      <c r="L47" s="37">
-        <f>K47*5</f>
-        <v>5</v>
-      </c>
-      <c r="M47" s="36"/>
-    </row>
-    <row r="48" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K47" s="60">
+        <v>4</v>
+      </c>
+      <c r="L47" s="39">
+        <f t="shared" ref="L47" si="18">K47*5</f>
+        <v>20</v>
+      </c>
+      <c r="M47" s="38"/>
+    </row>
+    <row r="48" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="56" t="s">
-        <v>19</v>
-      </c>
-      <c r="D48" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="E48" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="F48" s="38" t="s">
-        <v>142</v>
-      </c>
-      <c r="G48" s="39" t="s">
-        <v>182</v>
-      </c>
-      <c r="H48" s="64" t="s">
-        <v>210</v>
+      <c r="C48" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="E48" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="F48" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="G48" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H48" s="63" t="s">
+        <v>207</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J48" s="36"/>
-      <c r="K48" s="60">
+      <c r="K48" s="59">
         <v>1</v>
       </c>
-      <c r="L48" s="39">
-        <f t="shared" ref="L48" si="19">K48*5</f>
+      <c r="L48" s="37">
+        <f>K48*5</f>
         <v>5</v>
       </c>
-      <c r="M48" s="38"/>
+      <c r="M48" s="36"/>
     </row>
     <row r="49" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="50">
-        <f>ROW(B49) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="55" t="s">
-        <v>23</v>
-      </c>
-      <c r="D49" s="36" t="s">
-        <v>65</v>
-      </c>
-      <c r="E49" s="37" t="s">
-        <v>111</v>
-      </c>
-      <c r="F49" s="36" t="s">
-        <v>143</v>
-      </c>
-      <c r="G49" s="37" t="s">
-        <v>183</v>
-      </c>
-      <c r="H49" s="63" t="s">
-        <v>211</v>
+      <c r="C49" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="E49" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F49" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="G49" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="H49" s="64" t="s">
+        <v>209</v>
       </c>
       <c r="I49" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J49" s="36"/>
-      <c r="K49" s="59">
+      <c r="K49" s="60">
         <v>1</v>
       </c>
-      <c r="L49" s="37">
-        <f>K49*5</f>
+      <c r="L49" s="39">
+        <f t="shared" ref="L49" si="19">K49*5</f>
         <v>5</v>
       </c>
-      <c r="M49" s="36"/>
-    </row>
-    <row r="50" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M49" s="38"/>
+    </row>
+    <row r="50" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
-      <c r="C50" s="56" t="s">
+      <c r="C50" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="D50" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="E50" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="F50" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="G50" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="H50" s="64" t="s">
-        <v>211</v>
+      <c r="D50" s="36" t="s">
+        <v>64</v>
+      </c>
+      <c r="E50" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F50" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="G50" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="H50" s="63" t="s">
+        <v>210</v>
       </c>
       <c r="I50" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J50" s="36"/>
-      <c r="K50" s="60">
+      <c r="K50" s="59">
         <v>1</v>
       </c>
-      <c r="L50" s="39">
-        <f t="shared" ref="L50" si="20">K50*5</f>
+      <c r="L50" s="37">
+        <f>K50*5</f>
         <v>5</v>
       </c>
-      <c r="M50" s="38"/>
-    </row>
-    <row r="51" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M50" s="36"/>
+    </row>
+    <row r="51" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="50">
-        <f>ROW(B51) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="55" t="s">
-        <v>24</v>
-      </c>
-      <c r="D51" s="36" t="s">
-        <v>67</v>
-      </c>
-      <c r="E51" s="37" t="s">
-        <v>113</v>
-      </c>
-      <c r="F51" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="G51" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="H51" s="63" t="s">
-        <v>212</v>
+      <c r="C51" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="D51" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="E51" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="F51" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="G51" s="39" t="s">
+        <v>183</v>
+      </c>
+      <c r="H51" s="64" t="s">
+        <v>210</v>
       </c>
       <c r="I51" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J51" s="36"/>
-      <c r="K51" s="59">
+      <c r="K51" s="60">
         <v>1</v>
       </c>
-      <c r="L51" s="37">
-        <f>K51*5</f>
+      <c r="L51" s="39">
+        <f t="shared" ref="L51" si="20">K51*5</f>
         <v>5</v>
       </c>
-      <c r="M51" s="36"/>
-    </row>
-    <row r="52" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M51" s="38"/>
+    </row>
+    <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
-      <c r="C52" s="56" t="s">
-        <v>23</v>
-      </c>
-      <c r="D52" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="E52" s="39" t="s">
-        <v>114</v>
-      </c>
-      <c r="F52" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="G52" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="H52" s="64" t="s">
-        <v>213</v>
+      <c r="C52" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D52" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="E52" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="F52" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="G52" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="H52" s="63" t="s">
+        <v>211</v>
       </c>
       <c r="I52" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J52" s="36"/>
-      <c r="K52" s="60">
+      <c r="K52" s="59">
         <v>1</v>
       </c>
-      <c r="L52" s="39">
-        <f t="shared" ref="L52" si="21">K52*5</f>
+      <c r="L52" s="37">
+        <f>K52*5</f>
         <v>5</v>
       </c>
-      <c r="M52" s="38"/>
-    </row>
-    <row r="53" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M52" s="36"/>
+    </row>
+    <row r="53" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="50">
-        <f>ROW(B53) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C53" s="55" t="s">
+      <c r="C53" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="D53" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="E53" s="37" t="s">
-        <v>115</v>
-      </c>
-      <c r="F53" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="G53" s="37" t="s">
-        <v>187</v>
-      </c>
-      <c r="H53" s="63" t="s">
-        <v>214</v>
+      <c r="D53" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="E53" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="F53" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="G53" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="H53" s="64" t="s">
+        <v>212</v>
       </c>
       <c r="I53" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J53" s="36"/>
-      <c r="K53" s="59">
+      <c r="K53" s="60">
         <v>1</v>
       </c>
-      <c r="L53" s="37">
-        <f>K53*5</f>
+      <c r="L53" s="39">
+        <f t="shared" ref="L53" si="21">K53*5</f>
         <v>5</v>
       </c>
-      <c r="M53" s="36"/>
+      <c r="M53" s="38"/>
     </row>
     <row r="54" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
-      <c r="C54" s="56" t="s">
+      <c r="C54" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="D54" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="E54" s="39" t="s">
-        <v>116</v>
-      </c>
-      <c r="F54" s="38" t="s">
-        <v>148</v>
-      </c>
-      <c r="G54" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="H54" s="64" t="s">
-        <v>214</v>
+      <c r="D54" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="E54" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="F54" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="G54" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="H54" s="63" t="s">
+        <v>213</v>
       </c>
       <c r="I54" s="36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J54" s="36"/>
-      <c r="K54" s="60">
+      <c r="K54" s="59">
         <v>1</v>
       </c>
-      <c r="L54" s="39">
-        <f t="shared" ref="L54:L57" si="22">K54*5</f>
+      <c r="L54" s="37">
+        <f>K54*5</f>
         <v>5</v>
       </c>
-      <c r="M54" s="38"/>
+      <c r="M54" s="36"/>
     </row>
     <row r="55" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="50">
-        <f>ROW(B55) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C55" s="56" t="s">
-        <v>244</v>
+        <v>23</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>243</v>
+        <v>69</v>
       </c>
       <c r="E55" s="39" t="s">
-        <v>245</v>
+        <v>115</v>
       </c>
       <c r="F55" s="38" t="s">
-        <v>242</v>
+        <v>147</v>
       </c>
       <c r="G55" s="39" t="s">
-        <v>246</v>
-      </c>
-      <c r="H55" s="64"/>
-      <c r="I55" s="61"/>
+        <v>187</v>
+      </c>
+      <c r="H55" s="64" t="s">
+        <v>213</v>
+      </c>
+      <c r="I55" s="36" t="s">
+        <v>241</v>
+      </c>
       <c r="J55" s="36"/>
       <c r="K55" s="60">
         <v>1</v>
       </c>
       <c r="L55" s="39">
-        <f>K55*5</f>
+        <f t="shared" ref="L55:L58" si="22">K55*5</f>
         <v>5</v>
       </c>
       <c r="M55" s="38"/>
     </row>
-    <row r="56" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
-      <c r="C56" s="57" t="s">
-        <v>248</v>
+      <c r="C56" s="56" t="s">
+        <v>243</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E56" s="39" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="F56" s="38" t="s">
-        <v>242</v>
-      </c>
-      <c r="G56" s="38" t="s">
-        <v>242</v>
-      </c>
-      <c r="H56" s="39" t="s">
-        <v>242</v>
-      </c>
-      <c r="I56" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="J56" s="62" t="s">
-        <v>247</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="G56" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="H56" s="64"/>
+      <c r="I56" s="61"/>
+      <c r="J56" s="36"/>
       <c r="K56" s="60">
         <v>1</v>
       </c>
       <c r="L56" s="39">
-        <f t="shared" si="22"/>
+        <f>K56*5</f>
         <v>5</v>
       </c>
       <c r="M56" s="38"/>
@@ -3681,27 +3694,29 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C57" s="56" t="s">
-        <v>250</v>
+      <c r="C57" s="57" t="s">
+        <v>247</v>
       </c>
       <c r="D57" s="38" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E57" s="39" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F57" s="38" t="s">
-        <v>242</v>
-      </c>
-      <c r="G57" s="39" t="s">
-        <v>242</v>
-      </c>
-      <c r="H57" s="64" t="s">
-        <v>242</v>
-      </c>
-      <c r="I57" s="36"/>
+        <v>241</v>
+      </c>
+      <c r="G57" s="38" t="s">
+        <v>241</v>
+      </c>
+      <c r="H57" s="39" t="s">
+        <v>241</v>
+      </c>
+      <c r="I57" s="36" t="s">
+        <v>241</v>
+      </c>
       <c r="J57" s="62" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K57" s="60">
         <v>1</v>
@@ -3712,35 +3727,72 @@
       </c>
       <c r="M57" s="38"/>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
-      <c r="B58" s="31"/>
-      <c r="C58" s="48"/>
-      <c r="D58" s="32"/>
-      <c r="E58" s="33"/>
-      <c r="F58" s="34"/>
-      <c r="G58" s="35"/>
-      <c r="H58" s="34"/>
-      <c r="I58" s="35"/>
-      <c r="J58" s="35"/>
-      <c r="K58" s="35"/>
-      <c r="L58" s="35"/>
-      <c r="M58" s="41"/>
-    </row>
-    <row r="59" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="50">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="C58" s="56" t="s">
+        <v>249</v>
+      </c>
+      <c r="D58" s="38" t="s">
+        <v>242</v>
+      </c>
+      <c r="E58" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="F58" s="38" t="s">
+        <v>241</v>
+      </c>
+      <c r="G58" s="39" t="s">
+        <v>241</v>
+      </c>
+      <c r="H58" s="64" t="s">
+        <v>241</v>
+      </c>
+      <c r="I58" s="36"/>
+      <c r="J58" s="62" t="s">
+        <v>246</v>
+      </c>
+      <c r="K58" s="60">
+        <v>1</v>
+      </c>
+      <c r="L58" s="39">
+        <f t="shared" si="22"/>
+        <v>5</v>
+      </c>
+      <c r="M58" s="38"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="B59" s="24"/>
-      <c r="C59" s="49"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="9"/>
-      <c r="L59" s="9"/>
-      <c r="M59" s="42"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="48"/>
+      <c r="D59" s="32"/>
+      <c r="E59" s="33"/>
+      <c r="F59" s="34"/>
+      <c r="G59" s="35"/>
+      <c r="H59" s="34"/>
+      <c r="I59" s="35"/>
+      <c r="J59" s="35"/>
+      <c r="K59" s="35"/>
+      <c r="L59" s="35"/>
+      <c r="M59" s="41"/>
+    </row>
+    <row r="60" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1"/>
+      <c r="B60" s="24"/>
+      <c r="C60" s="49"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
+      <c r="I60" s="9"/>
+      <c r="J60" s="9"/>
+      <c r="K60" s="9"/>
+      <c r="L60" s="9"/>
+      <c r="M60" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3748,8 +3800,8 @@
     <mergeCell ref="M3:M8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J57" r:id="rId1"/>
-    <hyperlink ref="J56" r:id="rId2"/>
+    <hyperlink ref="J58" r:id="rId1"/>
+    <hyperlink ref="J57" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>